<commit_message>
Stage 8 fixes: G-010
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-19-S0100/Raw_Observations/VP10_Genotox_RESULTS_081919.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-19-S0100/Raw_Observations/VP10_Genotox_RESULTS_081919.xlsx
@@ -177,7 +177,7 @@
   <commentList>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Consistent across the mammalian readouts, so the side-chain concern goes into the summary to Valquessia as written.</t>
+        <t>Displayed Ames and micronucleus tables do not support the branch-drop genotoxicity rationale. Obtain the identified investigation/decision record under OQ/2019/001605; do not infer genotoxicity from viability loss.</t>
       </text>
     </comment>
   </commentList>
@@ -192,7 +192,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Dropping the branch is Valquessia's decision. Our part is to state the concern plainly.</t>
+        <t>Valquessia dropped the branch. These displayed negative results do not substantiate the genotoxicity rationale; identify the supporting investigation record before attributing it.</t>
       </text>
     </comment>
   </commentList>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -719,6 +719,31 @@
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t>USD 40,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Compliance status</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>GLP status is not documented in this endpoint summary. Consult the signed investigation plan and QA statement under OQ/2019/001605; no conclusion here is designated GLP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Decision provenance</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Branch-drop decision retained; supporting genotoxicity investigation identifier is not recorded here and must be established before citing a genotoxicity rationale.</t>
         </is>
       </c>
     </row>
@@ -749,7 +774,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>HepG2 viability screen (ATP content), 24 h and 48 h exposure. Investigation OT-19-S0100.</t>
+          <t>HepG2 viability screen (ATP content), 24 h and 48 h exposure. Cytotoxicity endpoint only; not a genotoxicity readout.</t>
         </is>
       </c>
     </row>
@@ -1344,14 +1369,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Bacterial mutation assay with and without S9. Mean revertants per plate, n=3. Fold is against the vehicle control on the same strain.</t>
+          <t>Bacterial mutation assay with and without S9; mean revertants/plate, n=3. The archived Fold vs vehicle column has an undocumented denominator: vehicle rows are not consistently unity. Do not interpret these values as folds over concurrent strain/activation-matched vehicle. Resolve the denominator from original calculation records under OQ/2019/001605 before using folds; values are retained unchanged.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Control validity met for every strain. Bacterial result is negative, as stated on the summary.</t>
+          <t>Reported bacterial outcome: negative. Control-validity details remain in original investigation records; fold-normalisation discrepancy is unresolved here.</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3154,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Side-chain concern: the signal repeats across the reactive analogues, not the parent series.</t>
+          <t>Displayed micronucleus result is negative, with values around vehicle levels. No analogue identifiers are provided in this table, so it cannot establish repeated effects across reactive analogues. Branch-drop rationale needs an identified source record.</t>
         </is>
       </c>
     </row>

</xml_diff>